<commit_message>
banch.xlsx: more measurements (as presented on 2024-12-04)
</commit_message>
<xml_diff>
--- a/bench.xlsx
+++ b/bench.xlsx
@@ -46,7 +46,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E12" authorId="1" xr:uid="{44FE1040-EA6E-1D7C-5CD3-EEAB189226D0}">
+    <comment ref="E13" authorId="1" xr:uid="{44FE1040-EA6E-1D7C-5CD3-EEAB189226D0}">
       <text>
         <r>
           <rPr>
@@ -117,12 +117,12 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={CA9AA1C9-6AD3-364A-9DC1-052A22FDB9B4}</author>
-    <author>tc={BDC83CEB-A7B1-AC8D-239A-6FEB488AC23E}</author>
-    <author>tc={10C544B4-EB2D-391F-CA6A-D49CF56E7AE9}</author>
+    <author>tc={FBA8A04F-1144-D4CE-3955-9139357F1DF7}</author>
+    <author>tc={49BA0359-1DD6-6E69-0623-10EC65534207}</author>
+    <author>tc={71B80EF3-EE31-C54E-AB34-BCEA6BB0C751}</author>
   </authors>
   <commentList>
-    <comment ref="A2" authorId="0" xr:uid="{CA9AA1C9-6AD3-364A-9DC1-052A22FDB9B4}">
+    <comment ref="A2" authorId="0" xr:uid="{FBA8A04F-1144-D4CE-3955-9139357F1DF7}">
       <text>
         <r>
           <rPr>
@@ -143,7 +143,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A3" authorId="1" xr:uid="{BDC83CEB-A7B1-AC8D-239A-6FEB488AC23E}">
+    <comment ref="A3" authorId="1" xr:uid="{49BA0359-1DD6-6E69-0623-10EC65534207}">
       <text>
         <r>
           <rPr>
@@ -164,7 +164,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A4" authorId="2" xr:uid="{10C544B4-EB2D-391F-CA6A-D49CF56E7AE9}">
+    <comment ref="A4" authorId="2" xr:uid="{71B80EF3-EE31-C54E-AB34-BCEA6BB0C751}">
       <text>
         <r>
           <rPr>
@@ -190,7 +190,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>stylegan3-r</t>
   </si>
@@ -204,25 +204,34 @@
     <t xml:space="preserve">&lt; source</t>
   </si>
   <si>
-    <t xml:space="preserve">A770 (XPU)</t>
+    <t xml:space="preserve">A770 (XPU, PyTorch 2.1.x)</t>
   </si>
   <si>
     <t xml:space="preserve">bench log 2024-12-03.html</t>
   </si>
   <si>
-    <t xml:space="preserve">PVC Max 1100 (XPU)</t>
+    <t xml:space="preserve">PVC Max 1100 (XPU, PyTorch 2.1.x)</t>
   </si>
   <si>
     <t xml:space="preserve">Intel PVC VM stylegan3 more speed measurements (before+after the 5x speedup commit and -01 vs -O3) 2024-11-21.txt</t>
   </si>
   <si>
-    <t xml:space="preserve">1080Ti (CUDA)</t>
+    <t xml:space="preserve">1080Ti (CUDA, PyTorch 1.9.1)</t>
   </si>
   <si>
-    <t xml:space="preserve">A770 ("ref")</t>
+    <t xml:space="preserve">1080Ti (CUDA, PyTorch 2.1.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bench log 2024-12-04.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A770 ("ref", PyTorch 2.1.x)</t>
   </si>
   <si>
     <t xml:space="preserve">1080Ti ("ref", PyTorch 1.9.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1080Ti ("ref", PyTorch 2.1.2)</t>
   </si>
   <si>
     <t xml:space="preserve">Notes: measured with "./bench3.sh" (gen_video.py with [network_variant]-afhqv2-512x512.pkl), always using the median value as the result</t>
@@ -246,7 +255,7 @@
     <t>2.1.40+xpu</t>
   </si>
   <si>
-    <t xml:space="preserve">1.9.1 (py3.9_cuda11.1_cudnn8.0.5_0)</t>
+    <t xml:space="preserve">1.9.1 (py3.9_cuda11.1_cudnn8.0.5_0), and later re-measured with 2.1.2 (py3.9_cuda12.1_cudnn8.9.2_0)</t>
   </si>
   <si>
     <t>driver</t>
@@ -268,6 +277,9 @@
   </si>
   <si>
     <t xml:space="preserve">CUDA Version: 12.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1080Ti (CUDA)</t>
   </si>
 </sst>
 </file>
@@ -418,7 +430,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>A770 (XPU)</c:v>
+                  <c:v>A770 (XPU, PyTorch 2.1.x)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -517,7 +529,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>PVC Max 1100 (XPU)</c:v>
+                  <c:v>PVC Max 1100 (XPU, PyTorch 2.1.x)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -616,7 +628,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>1080Ti (CUDA)</c:v>
+                  <c:v>1080Ti (CUDA, PyTorch 1.9.1)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -715,7 +727,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>A770 ("ref")</c:v>
+                  <c:v>1080Ti (CUDA, PyTorch 2.1.2)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -793,13 +805,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>1.01</c:v>
+                  <c:v>13.86</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.77</c:v>
+                  <c:v>7.04</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>24.52</c:v>
+                  <c:v>36.68</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -814,7 +826,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>1080Ti ("ref")</c:v>
+                  <c:v>A770 ("ref", PyTorch 2.1.x)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -892,6 +904,105 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>1.01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.77</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>24.52</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>current!$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>1080Ti ("ref", PyTorch 1.9.1)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr bwMode="auto">
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="accent6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:dLblPos val="outEnd"/>
+            <c:separator xml:space="preserve"> </c:separator>
+            <c:showBubbleSize val="0"/>
+            <c:showCatName val="0"/>
+            <c:showLegendKey val="0"/>
+            <c:showPercent val="0"/>
+            <c:showSerName val="0"/>
+            <c:showVal val="1"/>
+            <c:spPr bwMode="auto">
+              <a:prstGeom prst="rect">
+                <a:avLst/>
+              </a:prstGeom>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:txPr>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>current!$B$1:$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>stylegan3-r</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>stylegan3-t</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>stylegan2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>current!$B$7:$D$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
                   <c:v>0.24</c:v>
                 </c:pt>
                 <c:pt idx="1">
@@ -899,6 +1010,107 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>15.13</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>current!$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>1080Ti ("ref", PyTorch 2.1.2)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr bwMode="auto">
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="60000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:dLblPos val="outEnd"/>
+            <c:separator xml:space="preserve"> </c:separator>
+            <c:showBubbleSize val="0"/>
+            <c:showCatName val="0"/>
+            <c:showLegendKey val="0"/>
+            <c:showPercent val="0"/>
+            <c:showSerName val="0"/>
+            <c:showVal val="1"/>
+            <c:spPr bwMode="auto">
+              <a:prstGeom prst="rect">
+                <a:avLst/>
+              </a:prstGeom>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:txPr>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>current!$B$1:$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>stylegan3-r</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>stylegan3-t</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>stylegan2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>current!$B$8:$D$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>0.23</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.82</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>22.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -944,11 +1156,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-26"/>
-        <c:axId val="2140841633"/>
-        <c:axId val="2140841634"/>
+        <c:axId val="2140841721"/>
+        <c:axId val="2140841722"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2140841633"/>
+        <c:axId val="2140841721"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -992,7 +1204,7 @@
             <a:endParaRPr/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2140841634"/>
+        <c:crossAx val="2140841722"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1001,7 +1213,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2140841634"/>
+        <c:axId val="2140841722"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1027,7 +1239,7 @@
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="0" vert="horz"/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -1043,7 +1255,7 @@
           <c:layout/>
           <c:overlay val="0"/>
           <c:txPr>
-            <a:bodyPr/>
+            <a:bodyPr rot="0" vert="horz"/>
             <a:p>
               <a:pPr>
                 <a:defRPr/>
@@ -1084,7 +1296,7 @@
             <a:endParaRPr/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2140841633"/>
+        <c:crossAx val="2140841721"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1139,8 +1351,8 @@
   </c:chart>
   <c:spPr bwMode="auto">
     <a:xfrm rot="0" flipH="0" flipV="0">
-      <a:off x="4895849" y="314324"/>
-      <a:ext cx="6686549" cy="3681412"/>
+      <a:off x="6257924" y="1133474"/>
+      <a:ext cx="8124824" cy="4119562"/>
     </a:xfrm>
     <a:prstGeom prst="rect">
       <a:avLst/>
@@ -3009,27 +3221,27 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>361949</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>138112</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>371474</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>76199</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>342899</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>119062</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>571499</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>142874</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="197694986" name=""/>
+        <xdr:cNvPr id="370919270" name=""/>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm rot="0" flipH="0" flipV="0">
-        <a:off x="4895849" y="314324"/>
-        <a:ext cx="6686549" cy="3681412"/>
+        <a:off x="6257924" y="1133474"/>
+        <a:ext cx="8124824" cy="4119562"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3081,7 +3293,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="user" id="{AFCEB222-9418-A19C-68A0-D60362A1939D}" userId="user" providerId="Teamlab"/>
+  <person displayName="user" id="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" userId="user" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -3577,20 +3789,20 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A2" dT="2024-12-03T16:35:38.28Z" personId="{AFCEB222-9418-A19C-68A0-D60362A1939D}" id="{5D1DD697-3B31-24C3-D1FC-4F10BC94625B}" done="0">
+  <threadedComment ref="A2" dT="2024-12-03T16:35:38.28Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{5D1DD697-3B31-24C3-D1FC-4F10BC94625B}" done="0">
     <text xml:space="preserve">heads/debug_profiling-0-g9390a36 with "ENVNAME=stylegan3_2_1_40_xpu"
 </text>
   </threadedComment>
-  <threadedComment ref="E12" dT="2024-12-03T17:44:41.53Z" personId="{AFCEB222-9418-A19C-68A0-D60362A1939D}" id="{44FE1040-EA6E-1D7C-5CD3-EEAB189226D0}" done="0">
+  <threadedComment ref="E13" dT="2024-12-03T17:44:41.53Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{44FE1040-EA6E-1D7C-5CD3-EEAB189226D0}" done="1">
     <text xml:space="preserve">TODO try upgrading and re-measuring
 </text>
   </threadedComment>
-  <threadedComment ref="A3" dT="2024-12-03T16:08:51.51Z" personId="{AFCEB222-9418-A19C-68A0-D60362A1939D}" id="{9885B1C3-AB22-94B7-30B7-E8A667F23725}" done="0">
+  <threadedComment ref="A3" dT="2024-12-03T16:08:51.51Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{9885B1C3-AB22-94B7-30B7-E8A667F23725}" done="0">
     <text xml:space="preserve">9390a36a6b1ee05f376ece3fc065dfb77f459ded with "-O1" (which is in the commit)
 on a VM instance on Intel Tiber Developer Cloud
 </text>
   </threadedComment>
-  <threadedComment ref="A4" dT="2024-12-03T16:36:13.13Z" personId="{AFCEB222-9418-A19C-68A0-D60362A1939D}" id="{07C5CB9B-011A-F201-BE01-B6ED5DCC747A}" done="0">
+  <threadedComment ref="A4" dT="2024-12-03T16:36:13.13Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{07C5CB9B-011A-F201-BE01-B6ED5DCC747A}" done="0">
     <text xml:space="preserve">heads/debug_profiling-0-g9390a36 with "stylegan" environment
 </text>
   </threadedComment>
@@ -3599,15 +3811,15 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A2" dT="2024-12-03T16:35:38.28Z" personId="{AFCEB222-9418-A19C-68A0-D60362A1939D}" id="{CA9AA1C9-6AD3-364A-9DC1-052A22FDB9B4}" done="0">
+  <threadedComment ref="A2" dT="2024-12-03T16:35:38.28Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{FBA8A04F-1144-D4CE-3955-9139357F1DF7}" done="0">
     <text xml:space="preserve">heads/debug_profiling-0-g9390a36 with "ENVNAME=stylegan3_2_1_40_xpu"
 </text>
   </threadedComment>
-  <threadedComment ref="A3" dT="2024-12-03T16:08:51.51Z" personId="{AFCEB222-9418-A19C-68A0-D60362A1939D}" id="{BDC83CEB-A7B1-AC8D-239A-6FEB488AC23E}" done="0">
+  <threadedComment ref="A3" dT="2024-12-03T16:08:51.51Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{49BA0359-1DD6-6E69-0623-10EC65534207}" done="0">
     <text xml:space="preserve">9390a36a6b1ee05f376ece3fc065dfb77f459ded with "-O1" (which is in the commit)
 </text>
   </threadedComment>
-  <threadedComment ref="A4" dT="2024-12-03T16:36:13.13Z" personId="{AFCEB222-9418-A19C-68A0-D60362A1939D}" id="{10C544B4-EB2D-391F-CA6A-D49CF56E7AE9}" done="0">
+  <threadedComment ref="A4" dT="2024-12-03T16:36:13.13Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{71B80EF3-EE31-C54E-AB34-BCEA6BB0C751}" done="0">
     <text xml:space="preserve">heads/debug_profiling-0-g9390a36 with "stylegan" environment
 </text>
   </threadedComment>
@@ -3692,97 +3904,130 @@
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3">
-        <v>1.01</v>
-      </c>
-      <c r="C5" s="3">
-        <v>1.77</v>
-      </c>
-      <c r="D5" s="3">
-        <v>24.52</v>
+      <c r="B5" s="2">
+        <v>13.859999999999999</v>
+      </c>
+      <c r="C5" s="2">
+        <v>7.04</v>
+      </c>
+      <c r="D5" s="2">
+        <v>36.68</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6">
-        <v>0.23999999999999999</v>
-      </c>
-      <c r="C6">
-        <v>0.92000000000000004</v>
-      </c>
-      <c r="D6">
-        <v>15.130000000000001</v>
+      <c r="A6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1.01</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1.77</v>
+      </c>
+      <c r="D6" s="2">
+        <v>24.52</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" ht="14.25"/>
-    <row r="8" ht="14.25"/>
-    <row r="9" ht="14.25">
-      <c r="A9" t="s">
-        <v>11</v>
+    <row r="7" ht="14.25">
+      <c r="A7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <v>0.23999999999999999</v>
+      </c>
+      <c r="C7">
+        <v>0.92000000000000004</v>
+      </c>
+      <c r="D7">
+        <v>15.130000000000001</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="11" ht="14.25">
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
+    <row r="8" ht="14.25">
+      <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="E11" t="s">
+      <c r="B8">
+        <v>0.23000000000000001</v>
+      </c>
+      <c r="C8">
+        <v>0.81999999999999995</v>
+      </c>
+      <c r="D8">
+        <v>22.699999999999999</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="A10" t="s">
         <v>14</v>
       </c>
     </row>
+    <row r="11" ht="14.25"/>
     <row r="12" ht="14.25">
-      <c r="A12" t="s">
+      <c r="C12" t="s">
         <v>15</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
         <v>16</v>
       </c>
-      <c r="C12" t="s">
+      <c r="E12" t="s">
         <v>17</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="13" ht="14.25">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
       <c r="B13" t="s">
         <v>19</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" t="s">
         <v>21</v>
-      </c>
-      <c r="E13" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="14" ht="14.25">
       <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" t="s">
         <v>23</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>24</v>
       </c>
-      <c r="D14" t="s">
-        <v>21</v>
-      </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -3816,7 +4061,7 @@
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B2">
         <v>7.4500000000000002</v>
@@ -3830,7 +4075,7 @@
     </row>
     <row r="3" ht="14.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B3">
         <v>6.4199999999999999</v>
@@ -3844,7 +4089,7 @@
     </row>
     <row r="4" ht="14.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="B4">
         <v>11.9</v>
@@ -3858,7 +4103,7 @@
     </row>
     <row r="7" ht="14.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bench.xlsx: added relative speedups
</commit_message>
<xml_diff>
--- a/bench.xlsx
+++ b/bench.xlsx
@@ -190,7 +190,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>stylegan3-r</t>
   </si>
@@ -279,6 +279,21 @@
     <t xml:space="preserve">CUDA Version: 12.2</t>
   </si>
   <si>
+    <t xml:space="preserve">1080Ti (speedup "ref" -&gt; CUDA, PyTorch 1.9.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1080Ti (speedup "ref" -&gt; CUDA, PyTorch 2.1.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A770 (speedup "ref" -&gt; XPU, PyTorch 2.1.x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"ref" speedup A770 vs 1080Ti (PyTorch 2.1.x vs 1.9.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"ref" speedup A770 vs 1080Ti (PyTorch 2.1.x vs 2.1.2)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1080Ti (CUDA)</t>
   </si>
 </sst>
@@ -325,7 +340,9 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,6 +468,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -550,6 +568,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -649,6 +668,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -748,6 +768,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -847,6 +868,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -946,6 +968,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -1047,6 +1070,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -1121,6 +1145,7 @@
           <c:separator xml:space="preserve"> </c:separator>
           <c:showBubbleSize val="0"/>
           <c:showCatName val="0"/>
+          <c:showLeaderLines val="0"/>
           <c:showLegendKey val="0"/>
           <c:showPercent val="0"/>
           <c:showSerName val="0"/>
@@ -1351,7 +1376,7 @@
   </c:chart>
   <c:spPr bwMode="auto">
     <a:xfrm rot="0" flipH="0" flipV="0">
-      <a:off x="6257924" y="1133474"/>
+      <a:off x="6257923" y="1133474"/>
       <a:ext cx="8124824" cy="4119562"/>
     </a:xfrm>
     <a:prstGeom prst="rect">
@@ -1513,6 +1538,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -1613,6 +1639,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -1713,6 +1740,7 @@
             <c:separator xml:space="preserve"> </c:separator>
             <c:showBubbleSize val="0"/>
             <c:showCatName val="0"/>
+            <c:showLeaderLines val="0"/>
             <c:showLegendKey val="0"/>
             <c:showPercent val="0"/>
             <c:showSerName val="0"/>
@@ -1787,6 +1815,7 @@
           <c:separator xml:space="preserve"> </c:separator>
           <c:showBubbleSize val="0"/>
           <c:showCatName val="0"/>
+          <c:showLeaderLines val="0"/>
           <c:showLegendKey val="0"/>
           <c:showPercent val="0"/>
           <c:showSerName val="0"/>
@@ -3222,7 +3251,7 @@
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>371474</xdr:colOff>
+      <xdr:colOff>371473</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>76199</xdr:rowOff>
     </xdr:from>
@@ -3240,7 +3269,7 @@
         </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm rot="0" flipH="0" flipV="0">
-        <a:off x="6257924" y="1133474"/>
+        <a:off x="6257923" y="1133474"/>
         <a:ext cx="8124824" cy="4119562"/>
       </xdr:xfrm>
       <a:graphic>
@@ -3261,7 +3290,7 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>114299</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>66674</xdr:rowOff>
+      <xdr:rowOff>66673</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
@@ -3293,7 +3322,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="user" id="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" userId="user" providerId="Teamlab"/>
+  <person displayName="user" id="{D8426B48-3D18-4E14-7890-79335D173E8D}" userId="user" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -3789,20 +3818,20 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A2" dT="2024-12-03T16:35:38.28Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{5D1DD697-3B31-24C3-D1FC-4F10BC94625B}" done="0">
+  <threadedComment ref="A2" dT="2024-12-03T16:35:38.28Z" personId="{D8426B48-3D18-4E14-7890-79335D173E8D}" id="{5D1DD697-3B31-24C3-D1FC-4F10BC94625B}" done="0">
     <text xml:space="preserve">heads/debug_profiling-0-g9390a36 with "ENVNAME=stylegan3_2_1_40_xpu"
 </text>
   </threadedComment>
-  <threadedComment ref="E13" dT="2024-12-03T17:44:41.53Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{44FE1040-EA6E-1D7C-5CD3-EEAB189226D0}" done="1">
+  <threadedComment ref="E13" dT="2024-12-03T17:44:41.53Z" personId="{D8426B48-3D18-4E14-7890-79335D173E8D}" id="{44FE1040-EA6E-1D7C-5CD3-EEAB189226D0}" done="1">
     <text xml:space="preserve">TODO try upgrading and re-measuring
 </text>
   </threadedComment>
-  <threadedComment ref="A3" dT="2024-12-03T16:08:51.51Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{9885B1C3-AB22-94B7-30B7-E8A667F23725}" done="0">
+  <threadedComment ref="A3" dT="2024-12-03T16:08:51.51Z" personId="{D8426B48-3D18-4E14-7890-79335D173E8D}" id="{9885B1C3-AB22-94B7-30B7-E8A667F23725}" done="0">
     <text xml:space="preserve">9390a36a6b1ee05f376ece3fc065dfb77f459ded with "-O1" (which is in the commit)
 on a VM instance on Intel Tiber Developer Cloud
 </text>
   </threadedComment>
-  <threadedComment ref="A4" dT="2024-12-03T16:36:13.13Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{07C5CB9B-011A-F201-BE01-B6ED5DCC747A}" done="0">
+  <threadedComment ref="A4" dT="2024-12-03T16:36:13.13Z" personId="{D8426B48-3D18-4E14-7890-79335D173E8D}" id="{07C5CB9B-011A-F201-BE01-B6ED5DCC747A}" done="0">
     <text xml:space="preserve">heads/debug_profiling-0-g9390a36 with "stylegan" environment
 </text>
   </threadedComment>
@@ -3811,15 +3840,15 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A2" dT="2024-12-03T16:35:38.28Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{FBA8A04F-1144-D4CE-3955-9139357F1DF7}" done="0">
+  <threadedComment ref="A2" dT="2024-12-03T16:35:38.28Z" personId="{D8426B48-3D18-4E14-7890-79335D173E8D}" id="{FBA8A04F-1144-D4CE-3955-9139357F1DF7}" done="0">
     <text xml:space="preserve">heads/debug_profiling-0-g9390a36 with "ENVNAME=stylegan3_2_1_40_xpu"
 </text>
   </threadedComment>
-  <threadedComment ref="A3" dT="2024-12-03T16:08:51.51Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{49BA0359-1DD6-6E69-0623-10EC65534207}" done="0">
+  <threadedComment ref="A3" dT="2024-12-03T16:08:51.51Z" personId="{D8426B48-3D18-4E14-7890-79335D173E8D}" id="{49BA0359-1DD6-6E69-0623-10EC65534207}" done="0">
     <text xml:space="preserve">9390a36a6b1ee05f376ece3fc065dfb77f459ded with "-O1" (which is in the commit)
 </text>
   </threadedComment>
-  <threadedComment ref="A4" dT="2024-12-03T16:36:13.13Z" personId="{2273A713-94E1-773E-E6FE-AFA954FF6CEB}" id="{71B80EF3-EE31-C54E-AB34-BCEA6BB0C751}" done="0">
+  <threadedComment ref="A4" dT="2024-12-03T16:36:13.13Z" personId="{D8426B48-3D18-4E14-7890-79335D173E8D}" id="{71B80EF3-EE31-C54E-AB34-BCEA6BB0C751}" done="0">
     <text xml:space="preserve">heads/debug_profiling-0-g9390a36 with "stylegan" environment
 </text>
   </threadedComment>
@@ -3830,7 +3859,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="13.28125"/>
+    <col customWidth="1" min="1" max="1" width="32.28125"/>
     <col customWidth="1" min="2" max="3" width="12.140625"/>
     <col customWidth="1" min="4" max="4" width="14.140625"/>
   </cols>
@@ -3918,7 +3947,7 @@
       </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="2">
@@ -3935,7 +3964,7 @@
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B7">
@@ -3995,7 +4024,7 @@
       <c r="C13" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E13" t="s">
@@ -4026,8 +4055,53 @@
       <c r="D15" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="2" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="A22" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22">
+        <f>C4/C7</f>
+        <v>11.163043478260869</v>
+      </c>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="A23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23">
+        <f>C5/C8</f>
+        <v>8.5853658536585371</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24">
+        <f>C2/C6</f>
+        <v>5.6553672316384178</v>
+      </c>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27">
+        <f>C6/C7</f>
+        <v>1.9239130434782608</v>
+      </c>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="A28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28">
+        <f>C6/C8</f>
+        <v>2.1585365853658538</v>
       </c>
     </row>
   </sheetData>
@@ -4089,7 +4163,7 @@
     </row>
     <row r="4" ht="14.25">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B4">
         <v>11.9</v>

</xml_diff>